<commit_message>
Add CA broad campaign IDs to PD LTSF ID list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Wv13KPDszSjtnJt4JhRwx
</commit_message>
<xml_diff>
--- a/PD_LTSF_Campaign_IDs.xlsx
+++ b/PD_LTSF_Campaign_IDs.xlsx
@@ -915,7 +915,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>IDs are the campaign IDs shown under each campaign name in the Amazon Ads console. Blank budgets were not visible in the screenshots.</t>
+          <t>IDs are the campaign IDs shown under each campaign name in the Amazon Ads console. Read from console screenshots; copy IDs straight from the console if exact characters matter (0 vs O). Blank budgets were not visible in the screenshots.</t>
         </is>
       </c>
     </row>
@@ -1048,9 +1048,9 @@
           <t>None</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Live. No portfolio</t>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Live. No portfolio (US and CA broads use LTSF - Prime Day)</t>
         </is>
       </c>
     </row>
@@ -1078,14 +1078,30 @@
           <t>DBS4-CA-SP-BROAD-(PD-LTSF)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>A0341573DSJH8X3WHS6U</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Oct 6, 2026</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>No end date</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>LTSF - Prime Day</t>
+        </is>
+      </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Not built yet</t>
+          <t>Live. Set end date to Oct 7</t>
         </is>
       </c>
     </row>
@@ -1134,9 +1150,9 @@
           <t>None</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Live. No portfolio</t>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Live. No portfolio (US and CA broads use LTSF - Prime Day)</t>
         </is>
       </c>
     </row>
@@ -1164,14 +1180,30 @@
           <t>DBS6-CA-SP-BROAD-(PD-LTSF)</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>A01761552PZEMLSRQQZ9Q</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="n"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Oct 6, 2026</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>No end date</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>LTSF - Prime Day</t>
+        </is>
+      </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Not built yet</t>
+          <t>Live. Set end date to Oct 7</t>
         </is>
       </c>
     </row>
@@ -1220,9 +1252,9 @@
           <t>None</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Live. No portfolio. Check ID: 0 (zero) or O after "AD"</t>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Live. No portfolio (US and CA broads use LTSF - Prime Day)</t>
         </is>
       </c>
     </row>
@@ -1250,14 +1282,30 @@
           <t>DSS4-CA-SP-BROAD-(PD-LTSF)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>A0634724706FIL0SM12T</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Oct 6, 2026</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>No end date</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>LTSF - Prime Day</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Not built yet</t>
+          <t>Live. Set end date to Oct 7</t>
         </is>
       </c>
     </row>
@@ -1306,9 +1354,9 @@
           <t>None</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>Live. No portfolio</t>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Live. No portfolio (US and CA broads use LTSF - Prime Day)</t>
         </is>
       </c>
     </row>
@@ -1336,21 +1384,37 @@
           <t>DSS6-CA-SP-BROAD-(PD-LTSF)</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>A082665324UWVWP3TS7JU</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Oct 6, 2026</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>No end date</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>LTSF - Prime Day</t>
+        </is>
+      </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Not built yet</t>
+          <t>Live. Set end date to Oct 7</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>IDs are the campaign IDs shown under each campaign name in the Amazon Ads console. Blank budgets were not visible in the screenshots.</t>
+          <t>IDs are the campaign IDs shown under each campaign name in the Amazon Ads console. Read from console screenshots; copy IDs straight from the console if exact characters matter (0 vs O). Blank budgets were not visible in the screenshots.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add US Satin 4pc and Silk broad campaign IDs; all 16 PD LTSF IDs listed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Wv13KPDszSjtnJt4JhRwx
</commit_message>
<xml_diff>
--- a/PD_LTSF_Campaign_IDs.xlsx
+++ b/PD_LTSF_Campaign_IDs.xlsx
@@ -811,14 +811,30 @@
           <t>DSS4-SP-BROAD-(PD-LTSF)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>A04346875IOS06T3WX8Q</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Oct 6, 2026</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Check (not in screenshot)</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Check (not in screenshot)</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Not built yet</t>
+          <t>Live. Confirm end date Oct 7</t>
         </is>
       </c>
     </row>
@@ -901,14 +917,30 @@
           <t>D-SPC-SP-BROAD-(PD-LTSF)</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>A1036874NI3SYWYEGOAJ</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Oct 6, 2026</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Check (not in screenshot)</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Check (not in screenshot)</t>
+        </is>
+      </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Not built yet</t>
+          <t>Live. Confirm end date Oct 7</t>
         </is>
       </c>
     </row>

</xml_diff>